<commit_message>
Add NJ and CT car wash leads (17 new leads, 35 total)
New tabs: NJ Car Wash Leads (9) and CT Car Wash Leads (8).
Includes confirmed owner emails for CWONJ officers and other independents.
</commit_message>
<xml_diff>
--- a/NY_CarWash_Leads.xlsx
+++ b/NY_CarWash_Leads.xlsx
@@ -9,9 +9,13 @@
   <sheets>
     <sheet name="NY Car Wash Leads" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Summary &amp; Next Steps" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="NJ Car Wash Leads" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="CT Car Wash Leads" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'NY Car Wash Leads'!$A$1:$M$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'NJ Car Wash Leads'!$A$1:$M$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CT Car Wash Leads'!$A$1:$M$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -49,8 +53,14 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001A5276"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -72,8 +82,23 @@
         <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A5276"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6EAF8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D5F5E3"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -95,11 +120,25 @@
         <color rgb="00B0C4DE"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00AED6F1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00AED6F1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AED6F1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AED6F1"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -120,6 +159,21 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1790,7 +1844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -2009,7 +2063,1494 @@
         </is>
       </c>
     </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>NEW JERSEY — Key Stats</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Total NJ Leads:</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Confirmed NJ Emails:</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>dinodnico@gmail.com, dan@premiercarwashnj.com, hotwax100@hotmail.com, drieck@gmail.com, proshine93@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Hottest NJ Leads:</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Dino Nicoletta (CWONJ President), Dan Saidel (VP), Mike Prudente (Treasurer) — all industry insiders with confirmed emails</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="6" t="inlineStr"/>
+      <c r="B26" s="7" t="inlineStr"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>CONNECTICUT — Key Stats</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr"/>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>Total CT Leads:</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Confirmed CT Emails:</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>budgetcarwash@aol.com (Budget CW West Haven), info@wehawashes.com (WeHa Washes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Hottest CT Leads:</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Sammy Rivera (Budget CW, 30 yrs), Mark Lightowler (Buggy CW, 25 yrs), Tunji Somma (CT Auto Spa)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="6" t="inlineStr"/>
+      <c r="B31" s="7" t="inlineStr"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>RESOURCES — NJ &amp; CT</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr"/>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>Car Wash Operators of NJ (CWONJ)</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>cwonj.com — Exec Dir: Suzanne Stansbury | (518) 280-4767 | suzanne.stansbury@icloud.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>NJ DEP Car Wash List (PDF)</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>dep.nj.gov/wp-content/uploads/cleanwaternj/car_wash_list.pdf — full statewide list</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>Ross Brothers NJ/CT Broker</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>mycarwashbroker.com/new-jersey-car-wash-listings/ | mycarwashbroker.com/ctpa-car-wash-listings/</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>CT DAS Car Wash List (PDF)</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>portal.ct.gov — full CT state car wash list with vendor contacts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="001A5276"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="52" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Business Name</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>Owner / Contact Name</t>
+        </is>
+      </c>
+      <c r="C1" s="9" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="D1" s="9" t="inlineStr">
+        <is>
+          <t>Region / County</t>
+        </is>
+      </c>
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="F1" s="9" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="G1" s="9" t="inlineStr">
+        <is>
+          <t>ZIP</t>
+        </is>
+      </c>
+      <c r="H1" s="9" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="I1" s="9" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="J1" s="9" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="K1" s="9" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="L1" s="9" t="inlineStr">
+        <is>
+          <t>Notes / Status</t>
+        </is>
+      </c>
+      <c r="M1" s="9" t="inlineStr">
+        <is>
+          <t>Franchise? (Y/N)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Asbury Circle Car Wash</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
+          <t>Dino Nicoletta (Owner / CWONJ President)</t>
+        </is>
+      </c>
+      <c r="C2" s="10" t="inlineStr">
+        <is>
+          <t>707 NJ-35</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="inlineStr">
+        <is>
+          <t>Monmouth County</t>
+        </is>
+      </c>
+      <c r="E2" s="10" t="inlineStr">
+        <is>
+          <t>Neptune</t>
+        </is>
+      </c>
+      <c r="F2" s="10" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="G2" s="10" t="inlineStr">
+        <is>
+          <t>07753</t>
+        </is>
+      </c>
+      <c r="H2" s="10" t="inlineStr">
+        <is>
+          <t>(732) 455-3618</t>
+        </is>
+      </c>
+      <c r="I2" s="10" t="inlineStr">
+        <is>
+          <t>dinodnico@gmail.com</t>
+        </is>
+      </c>
+      <c r="J2" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K2" s="10" t="inlineStr">
+        <is>
+          <t>Full-Service / Automated</t>
+        </is>
+      </c>
+      <c r="L2" s="10" t="inlineStr">
+        <is>
+          <t>In industry since 1995; previously owned City Line Car Wash JC &amp; Shrewsbury CW. CWONJ President. Very connected — excellent relationship lead.</t>
+        </is>
+      </c>
+      <c r="M2" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="40" customHeight="1">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>Premier Car Wash</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>Dan Saidel (Owner / CWONJ Vice President)</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="inlineStr">
+        <is>
+          <t>175 Essex Ave</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>Middlesex County</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>Metuchen</t>
+        </is>
+      </c>
+      <c r="F3" s="11" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="G3" s="11" t="inlineStr">
+        <is>
+          <t>08840</t>
+        </is>
+      </c>
+      <c r="H3" s="11" t="inlineStr">
+        <is>
+          <t>(201) 736-9926</t>
+        </is>
+      </c>
+      <c r="I3" s="11" t="inlineStr">
+        <is>
+          <t>dan@premiercarwashnj.com</t>
+        </is>
+      </c>
+      <c r="J3" s="11" t="inlineStr">
+        <is>
+          <t>premiercarwashnj.com</t>
+        </is>
+      </c>
+      <c r="K3" s="11" t="inlineStr">
+        <is>
+          <t>Full-Service</t>
+        </is>
+      </c>
+      <c r="L3" s="11" t="inlineStr">
+        <is>
+          <t>VP of CWONJ; verified email. Strong acquisition/expansion target.</t>
+        </is>
+      </c>
+      <c r="M3" s="11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="40" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Summit Car Wash &amp; Detail Center</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Mike Prudente (Owner / CWONJ Treasurer)</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>100 Springfield Ave</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>Union County</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>Summit</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>07901</t>
+        </is>
+      </c>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>(908) 273-0830</t>
+        </is>
+      </c>
+      <c r="I4" s="10" t="inlineStr">
+        <is>
+          <t>hotwax100@hotmail.com</t>
+        </is>
+      </c>
+      <c r="J4" s="10" t="inlineStr">
+        <is>
+          <t>summitcarwash.20m.com</t>
+        </is>
+      </c>
+      <c r="K4" s="10" t="inlineStr">
+        <is>
+          <t>Full-Service / Detail</t>
+        </is>
+      </c>
+      <c r="L4" s="10" t="inlineStr">
+        <is>
+          <t>CWONJ Treasurer; confirmed email. May be open to exit or expansion conversation.</t>
+        </is>
+      </c>
+      <c r="M4" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>Manahawkin Magic Wash</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Doug Rieck (Owner)</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>578 Mill Creek Rd</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>Ocean County</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>Manahawkin</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>08050</t>
+        </is>
+      </c>
+      <c r="H5" s="11" t="inlineStr">
+        <is>
+          <t>(609) 597-7837</t>
+        </is>
+      </c>
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>drieck@gmail.com</t>
+        </is>
+      </c>
+      <c r="J5" s="11" t="inlineStr">
+        <is>
+          <t>manahawkinmagicwash.com</t>
+        </is>
+      </c>
+      <c r="K5" s="11" t="inlineStr">
+        <is>
+          <t>Self-Service / Coin-Op</t>
+        </is>
+      </c>
+      <c r="L5" s="11" t="inlineStr">
+        <is>
+          <t>Multiple locations (Waretown &amp; Pemberton also). Owner email confirmed. CWONJ board member.</t>
+        </is>
+      </c>
+      <c r="M5" s="11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>ProShine Hand Car Wash &amp; Detailing Center</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Wil &amp; Cynthia (Co-Owners)</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>93 State Route 35</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>Monmouth County</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>Eatontown</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>07724</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>(732) 544-2044</t>
+        </is>
+      </c>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t>proshine93@gmail.com</t>
+        </is>
+      </c>
+      <c r="J6" s="10" t="inlineStr">
+        <is>
+          <t>proshinehandcarwash.com</t>
+        </is>
+      </c>
+      <c r="K6" s="10" t="inlineStr">
+        <is>
+          <t>Hand Wash / Detail</t>
+        </is>
+      </c>
+      <c r="L6" s="10" t="inlineStr">
+        <is>
+          <t>Family-owned since 2017; owner email confirmed. Strong candidate.</t>
+        </is>
+      </c>
+      <c r="M6" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>Jersey Shine &amp; Lube LLC</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Tom &amp; Joe (Owners — family-run since 2004)</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>169 Route 70</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>Burlington County</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>Medford</t>
+        </is>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>08055</t>
+        </is>
+      </c>
+      <c r="H7" s="11" t="inlineStr">
+        <is>
+          <t>(609) 714-0940</t>
+        </is>
+      </c>
+      <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>Via jerseyshineandlube.com/contact</t>
+        </is>
+      </c>
+      <c r="J7" s="11" t="inlineStr">
+        <is>
+          <t>jerseyshineandlube.com</t>
+        </is>
+      </c>
+      <c r="K7" s="11" t="inlineStr">
+        <is>
+          <t>Full-Service / Lube</t>
+        </is>
+      </c>
+      <c r="L7" s="11" t="inlineStr">
+        <is>
+          <t>Family business 20+ years. Ask for Tom or Joe directly.</t>
+        </is>
+      </c>
+      <c r="M7" s="11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Kleen Kar Car Wash (multi-location)</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>John Laspata (Owner)</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>497 Williamstown Rd</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>Camden County</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>Sicklerville</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>08081</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>(856) 318-1361</t>
+        </is>
+      </c>
+      <c r="I8" s="10" t="inlineStr">
+        <is>
+          <t>Via kleenkarcarwash.com (ZoomInfo confirms email exists)</t>
+        </is>
+      </c>
+      <c r="J8" s="10" t="inlineStr">
+        <is>
+          <t>kleenkarcarwash.com</t>
+        </is>
+      </c>
+      <c r="K8" s="10" t="inlineStr">
+        <is>
+          <t>Tunnel / Automated</t>
+        </is>
+      </c>
+      <c r="L8" s="10" t="inlineStr">
+        <is>
+          <t>4 locations in South Jersey. Owner name confirmed via ZoomInfo. Expansion-minded operator.</t>
+        </is>
+      </c>
+      <c r="M8" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="40" customHeight="1">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>Jersey Auto Spa Car Wash &amp; Detail Center</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Mike (Manager / possible owner)</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Oceanport Ave</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>Monmouth County</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>West Long Branch</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>07764</t>
+        </is>
+      </c>
+      <c r="H9" s="11" t="inlineStr">
+        <is>
+          <t>Call to confirm</t>
+        </is>
+      </c>
+      <c r="I9" s="11" t="inlineStr">
+        <is>
+          <t>N/A — call to request</t>
+        </is>
+      </c>
+      <c r="J9" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K9" s="11" t="inlineStr">
+        <is>
+          <t>Full-Service / Detail</t>
+        </is>
+      </c>
+      <c r="L9" s="11" t="inlineStr">
+        <is>
+          <t>Independently run; confirm owner vs. manager status on call.</t>
+        </is>
+      </c>
+      <c r="M9" s="11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="40" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Ride and Shine Detail</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Greg &amp; Jack (Brothers / Co-Owners)</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>3 Westminster Pl</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>Bergen County</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>Garfield</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>07026</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>Call to confirm</t>
+        </is>
+      </c>
+      <c r="I10" s="10" t="inlineStr">
+        <is>
+          <t>Via rideshinedetail.com</t>
+        </is>
+      </c>
+      <c r="J10" s="10" t="inlineStr">
+        <is>
+          <t>rideshinedetail.com</t>
+        </is>
+      </c>
+      <c r="K10" s="10" t="inlineStr">
+        <is>
+          <t>Mobile / Detail</t>
+        </is>
+      </c>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>Family-owned brothers duo. Mobile operator — may want brick-and-mortar expansion.</t>
+        </is>
+      </c>
+      <c r="M10" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:M10"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00117A65"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="52" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Business Name</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>Owner / Contact Name</t>
+        </is>
+      </c>
+      <c r="C1" s="9" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="D1" s="9" t="inlineStr">
+        <is>
+          <t>Region / County</t>
+        </is>
+      </c>
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="F1" s="9" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="G1" s="9" t="inlineStr">
+        <is>
+          <t>ZIP</t>
+        </is>
+      </c>
+      <c r="H1" s="9" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="I1" s="9" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="J1" s="9" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="K1" s="9" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="L1" s="9" t="inlineStr">
+        <is>
+          <t>Notes / Status</t>
+        </is>
+      </c>
+      <c r="M1" s="9" t="inlineStr">
+        <is>
+          <t>Franchise? (Y/N)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Budget Car Wash LLC</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>Sammy Rivera (Owner)</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>936 Boston Post Rd</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
+        <is>
+          <t>New Haven County</t>
+        </is>
+      </c>
+      <c r="E2" s="12" t="inlineStr">
+        <is>
+          <t>West Haven</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="G2" s="12" t="inlineStr">
+        <is>
+          <t>06516</t>
+        </is>
+      </c>
+      <c r="H2" s="12" t="inlineStr">
+        <is>
+          <t>(203) 500-6149</t>
+        </is>
+      </c>
+      <c r="I2" s="12" t="inlineStr">
+        <is>
+          <t>budgetcarwash@aol.com</t>
+        </is>
+      </c>
+      <c r="J2" s="12" t="inlineStr">
+        <is>
+          <t>mybudgetcarwash.com</t>
+        </is>
+      </c>
+      <c r="K2" s="12" t="inlineStr">
+        <is>
+          <t>Express / Self-Service</t>
+        </is>
+      </c>
+      <c r="L2" s="12" t="inlineStr">
+        <is>
+          <t>Family-owned 30+ years. Owner name &amp; email confirmed. Strong acquisition/exit candidate.</t>
+        </is>
+      </c>
+      <c r="M2" s="12" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="40" customHeight="1">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>Buggy Car Wash</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>Mark Lightowler (Owner — since Sept 2000)</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="inlineStr">
+        <is>
+          <t>51 Middletown Ave</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>New Haven County</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>North Haven</t>
+        </is>
+      </c>
+      <c r="F3" s="11" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="G3" s="11" t="inlineStr">
+        <is>
+          <t>06473</t>
+        </is>
+      </c>
+      <c r="H3" s="11" t="inlineStr">
+        <is>
+          <t>(203) 495-9945</t>
+        </is>
+      </c>
+      <c r="I3" s="11" t="inlineStr">
+        <is>
+          <t>Via buggycarwash.com/contact-us</t>
+        </is>
+      </c>
+      <c r="J3" s="11" t="inlineStr">
+        <is>
+          <t>buggycarwash.com</t>
+        </is>
+      </c>
+      <c r="K3" s="11" t="inlineStr">
+        <is>
+          <t>Full-Service / Car &amp; Dog Wash</t>
+        </is>
+      </c>
+      <c r="L3" s="11" t="inlineStr">
+        <is>
+          <t>Family-owned 25+ years. Unique niche (dog wash). Owner name confirmed.</t>
+        </is>
+      </c>
+      <c r="M3" s="11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="40" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>CT Auto Spa LLC</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>Tunji Somma (Member / Owner)</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>39 Albany Tpke</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>Hartford County</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>West Simsbury</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="G4" s="12" t="inlineStr">
+        <is>
+          <t>06092</t>
+        </is>
+      </c>
+      <c r="H4" s="12" t="inlineStr">
+        <is>
+          <t>Call to confirm</t>
+        </is>
+      </c>
+      <c r="I4" s="12" t="inlineStr">
+        <is>
+          <t>Via ctautospa.com/contact</t>
+        </is>
+      </c>
+      <c r="J4" s="12" t="inlineStr">
+        <is>
+          <t>ctautospa.com</t>
+        </is>
+      </c>
+      <c r="K4" s="12" t="inlineStr">
+        <is>
+          <t>Full-Service / Detail</t>
+        </is>
+      </c>
+      <c r="L4" s="12" t="inlineStr">
+        <is>
+          <t>LLC; owner name confirmed via BBB. Farmington Valley's newest car wash — expansion minded.</t>
+        </is>
+      </c>
+      <c r="M4" s="12" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>Happy Hand Car Wash</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Unknown — call to verify</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>454 Stillson Rd</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>New Haven County</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>Waterbury</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>06705</t>
+        </is>
+      </c>
+      <c r="H5" s="11" t="inlineStr">
+        <is>
+          <t>(203) 528-3749</t>
+        </is>
+      </c>
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>N/A — call to request</t>
+        </is>
+      </c>
+      <c r="J5" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K5" s="11" t="inlineStr">
+        <is>
+          <t>Hand Wash</t>
+        </is>
+      </c>
+      <c r="L5" s="11" t="inlineStr">
+        <is>
+          <t>Active independent in Waterbury market.</t>
+        </is>
+      </c>
+      <c r="M5" s="11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Personal Touch Car Wash (True Blue Personal Touch LLC)</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>Unknown (Vincent Porzio Jr. linked to brand)</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>134 Thomaston Ave</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>New Haven County</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>Waterbury</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="inlineStr">
+        <is>
+          <t>06702</t>
+        </is>
+      </c>
+      <c r="H6" s="12" t="inlineStr">
+        <is>
+          <t>(203) 756-9311</t>
+        </is>
+      </c>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
+          <t>Via Facebook / call to request</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="inlineStr">
+        <is>
+          <t>personaltouchcarwashes.com</t>
+        </is>
+      </c>
+      <c r="K6" s="12" t="inlineStr">
+        <is>
+          <t>Express / Full-Service</t>
+        </is>
+      </c>
+      <c r="L6" s="12" t="inlineStr">
+        <is>
+          <t>LLC registered in CT; multiple locations under brand. Verify individual ownership.</t>
+        </is>
+      </c>
+      <c r="M6" s="12" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>WeHa Washes</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Unknown — student entrepreneur origin</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>West Hartford area</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>Hartford County</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>West Hartford</t>
+        </is>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>06107</t>
+        </is>
+      </c>
+      <c r="H7" s="11" t="inlineStr">
+        <is>
+          <t>(860) 558-8503</t>
+        </is>
+      </c>
+      <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>info@wehawashes.com</t>
+        </is>
+      </c>
+      <c r="J7" s="11" t="inlineStr">
+        <is>
+          <t>wehawashes.com</t>
+        </is>
+      </c>
+      <c r="K7" s="11" t="inlineStr">
+        <is>
+          <t>Mobile / Hand Wash</t>
+        </is>
+      </c>
+      <c r="L7" s="11" t="inlineStr">
+        <is>
+          <t>Local operator; email confirmed. May be interested in scaling up.</t>
+        </is>
+      </c>
+      <c r="M7" s="11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Platinum Car Wash &amp; Oil Change</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>Unknown — call to verify</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>1161 Wolcott St</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>New Haven County</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>Waterbury</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>06705</t>
+        </is>
+      </c>
+      <c r="H8" s="12" t="inlineStr">
+        <is>
+          <t>(203) 527-9700</t>
+        </is>
+      </c>
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>Via platinumcarwashandoil.com</t>
+        </is>
+      </c>
+      <c r="J8" s="12" t="inlineStr">
+        <is>
+          <t>platinumcarwashandoil.com</t>
+        </is>
+      </c>
+      <c r="K8" s="12" t="inlineStr">
+        <is>
+          <t>Full-Service / Lube</t>
+        </is>
+      </c>
+      <c r="L8" s="12" t="inlineStr">
+        <is>
+          <t>Independent operator; confirm owner on call.</t>
+        </is>
+      </c>
+      <c r="M8" s="12" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="40" customHeight="1">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>Turbo Clean Car Detailing</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Unknown — call to verify</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Waterbury area</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>New Haven County</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>Waterbury</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>06701</t>
+        </is>
+      </c>
+      <c r="H9" s="11" t="inlineStr">
+        <is>
+          <t>Call to confirm</t>
+        </is>
+      </c>
+      <c r="I9" s="11" t="inlineStr">
+        <is>
+          <t>Via turbocleanwaterbury.com</t>
+        </is>
+      </c>
+      <c r="J9" s="11" t="inlineStr">
+        <is>
+          <t>turbocleanwaterbury.com</t>
+        </is>
+      </c>
+      <c r="K9" s="11" t="inlineStr">
+        <is>
+          <t>Mobile / Detail</t>
+        </is>
+      </c>
+      <c r="L9" s="11" t="inlineStr">
+        <is>
+          <t>Serves New Haven, Stamford, Waterbury. Possible expansion candidate.</t>
+        </is>
+      </c>
+      <c r="M9" s="11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:M9"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>